<commit_message>
update Datenbank, update Auslesen Werte
</commit_message>
<xml_diff>
--- a/260513_Betonartikel/260506_Datenbankdefinition_Hochbau.xlsx
+++ b/260513_Betonartikel/260506_Datenbankdefinition_Hochbau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hodelan\PycharmProjects\StustainabilityDrivenStructuralDesign\260513_Betonartikel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C5EDC21-88C2-4263-A361-C0D156CCD57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CEAC507-BCD1-4B64-8B98-5BDCAE69EFDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-8850" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="clarification" sheetId="5" r:id="rId1"/>
@@ -40400,11 +40400,11 @@
         <v>6</v>
       </c>
       <c r="F5" s="23">
-        <v>2000</v>
+        <v>1450</v>
       </c>
       <c r="G5" s="23">
         <f t="shared" si="0"/>
-        <v>20000</v>
+        <v>14500</v>
       </c>
       <c r="H5" s="23">
         <v>1.7999999999999999E-2</v>

</xml_diff>